<commit_message>
chore(mappa): aggiornamento automatico 2026-07-02
</commit_message>
<xml_diff>
--- a/Milano_2027.xlsx
+++ b/Milano_2027.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\scarg\Dropbox\PNE Simone\Guide\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9AE74EB-58D5-4974-BC16-90F46887F634}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D34C2CC7-0FAC-459A-8194-3A03A58320FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="665" xr2:uid="{0118EB4B-1337-43BA-A7E3-0EBAC20BAF10}"/>
   </bookViews>
@@ -3848,15 +3848,15 @@
       </c>
       <c r="F4" s="9">
         <f>+AE6</f>
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G4" s="9">
         <f>+AG6</f>
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H4" s="7">
         <f>+E4-G4</f>
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I4" s="24" t="s">
         <v>16</v>
@@ -3878,15 +3878,15 @@
       </c>
       <c r="F5" s="11">
         <f>+F3+F4</f>
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G5" s="11">
         <f>+G3+G4</f>
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H5" s="11">
         <f>+H3+H4</f>
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I5" s="25" t="s">
         <v>43</v>
@@ -3979,7 +3979,7 @@
       </c>
       <c r="AE6" s="2">
         <f t="shared" si="1"/>
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="AF6" s="2">
         <f t="shared" si="1"/>
@@ -3987,7 +3987,7 @@
       </c>
       <c r="AG6" s="2">
         <f t="shared" si="1"/>
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="AH6" s="2">
         <f t="shared" si="1"/>
@@ -22788,51 +22788,53 @@
       </c>
     </row>
     <row r="175" spans="1:35" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A175" s="34">
-        <v>0</v>
-      </c>
-      <c r="B175" s="34">
+      <c r="A175" s="31">
+        <v>0</v>
+      </c>
+      <c r="B175" s="31">
         <v>2</v>
       </c>
-      <c r="C175" s="34">
+      <c r="C175" s="31">
         <v>4</v>
       </c>
-      <c r="D175" s="35" t="s">
+      <c r="D175" s="32" t="s">
         <v>62</v>
       </c>
-      <c r="E175" s="35" t="s">
+      <c r="E175" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="F175" s="35" t="s">
+      <c r="F175" s="32" t="s">
         <v>134</v>
       </c>
-      <c r="G175" s="35" t="s">
+      <c r="G175" s="32" t="s">
         <v>40</v>
       </c>
-      <c r="H175" s="35" t="s">
+      <c r="H175" s="32" t="s">
         <v>165</v>
       </c>
-      <c r="I175" s="34" t="s">
+      <c r="I175" s="31" t="s">
         <v>183</v>
       </c>
-      <c r="J175" s="34">
+      <c r="J175" s="31">
         <v>4</v>
       </c>
-      <c r="K175" s="34" t="s">
+      <c r="K175" s="31" t="s">
         <v>320</v>
       </c>
-      <c r="L175" s="34" t="s">
+      <c r="L175" s="31" t="s">
         <v>855</v>
       </c>
-      <c r="M175" s="35" t="s">
+      <c r="M175" s="32" t="s">
         <v>747</v>
       </c>
-      <c r="N175" s="35" t="s">
-        <v>931</v>
-      </c>
-      <c r="O175" s="36"/>
-      <c r="P175" s="36"/>
-      <c r="Q175" s="35"/>
+      <c r="N175" s="32" t="s">
+        <v>932</v>
+      </c>
+      <c r="O175" s="33">
+        <v>1</v>
+      </c>
+      <c r="P175" s="33"/>
+      <c r="Q175" s="32"/>
       <c r="S175" s="2">
         <f t="shared" si="51"/>
         <v>0</v>
@@ -22879,7 +22881,7 @@
       </c>
       <c r="AE175" s="2">
         <f t="shared" si="62"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF175" s="2">
         <f t="shared" si="47"/>
@@ -22887,7 +22889,7 @@
       </c>
       <c r="AG175" s="2">
         <f t="shared" si="48"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH175" s="2">
         <f t="shared" si="49"/>

</xml_diff>